<commit_message>
more experiments on weighted score
</commit_message>
<xml_diff>
--- a/weighted_score_exp.xlsx
+++ b/weighted_score_exp.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Model Stealing\tml2026-team_XLIII-assignment_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92E71DF4-4429-4FFB-B80F-AD1816A891E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7715D260-D1BB-45EF-89B2-58B926AF46E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{E8C8C0AA-81C6-4C35-80F1-F8A4E58A41C5}"/>
   </bookViews>
   <sheets>
     <sheet name="weighted_score_exp" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="21">
   <si>
     <t>Exp#</t>
   </si>
@@ -65,6 +78,24 @@
   </si>
   <si>
     <t>classifier-head-sensitive score</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>direct-copy detector</t>
+  </si>
+  <si>
+    <t>Max Score</t>
+  </si>
+  <si>
+    <t>Rank Based Average</t>
+  </si>
+  <si>
+    <t>weight-feature ensembles</t>
+  </si>
+  <si>
+    <t>classifier-head-dominant score</t>
   </si>
 </sst>
 </file>
@@ -554,7 +585,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -563,9 +594,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -943,7 +971,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F499B18-4DB0-44F6-A3C3-68C9F60D4845}">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -1050,7 +1078,7 @@
       <c r="K3" s="2">
         <v>0.05</v>
       </c>
-      <c r="M3" s="4">
+      <c r="M3" s="2">
         <v>0.53700000000000003</v>
       </c>
     </row>
@@ -1101,6 +1129,129 @@
       </c>
       <c r="K5" s="2">
         <v>0.1</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="K6" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K7" s="2">
+        <v>0.05</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0.05</v>
+      </c>
+      <c r="I11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J11" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="K11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
weighted score stage wise layers comparisons
</commit_message>
<xml_diff>
--- a/weighted_score_exp.xlsx
+++ b/weighted_score_exp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Model Stealing\tml2026-team_XLIII-assignment_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7715D260-D1BB-45EF-89B2-58B926AF46E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FADF0AB-CD23-4231-A46C-84E318F13CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{E8C8C0AA-81C6-4C35-80F1-F8A4E58A41C5}"/>
   </bookViews>
@@ -33,14 +33,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="31">
   <si>
     <t>Exp#</t>
   </si>
   <si>
-    <t>Importance</t>
-  </si>
-  <si>
     <t>mean_cosine</t>
   </si>
   <si>
@@ -96,6 +93,39 @@
   </si>
   <si>
     <t>classifier-head-dominant score</t>
+  </si>
+  <si>
+    <t>rank ensemble - rank</t>
+  </si>
+  <si>
+    <t>top evidence wins</t>
+  </si>
+  <si>
+    <t>v1_late_layers_fc</t>
+  </si>
+  <si>
+    <t>Not Increased</t>
+  </si>
+  <si>
+    <t>v2_fc_dominant_stage</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>v7_stage_rank_ensemble</t>
+  </si>
+  <si>
+    <t>v6_copy_or_partial_copy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v5_bn_sensitive  </t>
+  </si>
+  <si>
+    <t>v4_l2_plus_cosine</t>
+  </si>
+  <si>
+    <t>v3_backbone_progressive</t>
   </si>
 </sst>
 </file>
@@ -971,7 +1001,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F499B18-4DB0-44F6-A3C3-68C9F60D4845}">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
@@ -994,40 +1024,40 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -1061,7 +1091,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" s="2">
         <v>0.1</v>
@@ -1087,7 +1117,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C4" s="2">
         <v>0.25</v>
@@ -1113,7 +1143,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C5" s="2">
         <v>0.2</v>
@@ -1131,7 +1161,7 @@
         <v>0.1</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -1139,7 +1169,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C6" s="2">
         <v>0.2</v>
@@ -1154,7 +1184,7 @@
         <v>0.4</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -1162,7 +1192,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C7" s="2">
         <v>0.2</v>
@@ -1179,8 +1209,8 @@
       <c r="K7" s="2">
         <v>0.05</v>
       </c>
-      <c r="M7" s="1" t="s">
-        <v>15</v>
+      <c r="M7" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -1188,22 +1218,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -1211,10 +1241,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -1222,10 +1252,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -1233,7 +1263,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C11" s="2">
         <v>0.15</v>
@@ -1251,7 +1281,166 @@
         <v>0.1</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>15</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J12" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="K12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="G13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="H13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="K13" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="H14" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="J14" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="K14" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>1</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>2</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>3</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>4</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>5</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>6</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>7</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
more experiments of weighted score
</commit_message>
<xml_diff>
--- a/weighted_score_exp.xlsx
+++ b/weighted_score_exp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Model Stealing\tml2026-team_XLIII-assignment_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FADF0AB-CD23-4231-A46C-84E318F13CA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{573713C9-7194-4384-83CB-F5A46F692E21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{E8C8C0AA-81C6-4C35-80F1-F8A4E58A41C5}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="31">
   <si>
     <t>Exp#</t>
   </si>
@@ -1373,74 +1373,90 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B17" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>1</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>2</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>3</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>4</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>5</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>6</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>7</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
membership score experiment code
</commit_message>
<xml_diff>
--- a/weighted_score_exp.xlsx
+++ b/weighted_score_exp.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 2\tml2026-team_XLIII-assignment_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D9FE837-6EA6-401C-803D-1D746DD5C910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E44A68-7D9E-48C2-BE66-ED739C074B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{E8C8C0AA-81C6-4C35-80F1-F8A4E58A41C5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{E8C8C0AA-81C6-4C35-80F1-F8A4E58A41C5}"/>
   </bookViews>
   <sheets>
     <sheet name="weighted_score_exp" sheetId="1" r:id="rId1"/>
     <sheet name="output_behavior_score" sheetId="2" r:id="rId2"/>
+    <sheet name="membsership_score" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="49">
   <si>
     <t>Exp#</t>
   </si>
@@ -149,6 +150,36 @@
   </si>
   <si>
     <t>no change</t>
+  </si>
+  <si>
+    <t>loss_gap</t>
+  </si>
+  <si>
+    <t>confidence_gap</t>
+  </si>
+  <si>
+    <t>entropy_gap</t>
+  </si>
+  <si>
+    <t>margin_gap</t>
+  </si>
+  <si>
+    <t>accuracy_gap</t>
+  </si>
+  <si>
+    <t>gap_sim_loss</t>
+  </si>
+  <si>
+    <t>gap_sim_confidence</t>
+  </si>
+  <si>
+    <t>run id</t>
+  </si>
+  <si>
+    <t>leaderboard</t>
+  </si>
+  <si>
+    <t>notes</t>
   </si>
 </sst>
 </file>
@@ -638,7 +669,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -648,6 +679,9 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1610,4 +1644,84 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAB8347E-B43E-4F2F-85FC-E7ACB8853B0C}">
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="2" max="2" width="13.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" t="s">
+        <v>47</v>
+      </c>
+      <c r="J1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2">
+        <v>0.25</v>
+      </c>
+      <c r="B2">
+        <v>0.2</v>
+      </c>
+      <c r="C2">
+        <v>0.15</v>
+      </c>
+      <c r="D2">
+        <v>0.15</v>
+      </c>
+      <c r="E2">
+        <v>0.1</v>
+      </c>
+      <c r="F2">
+        <v>0.1</v>
+      </c>
+      <c r="G2">
+        <v>0.05</v>
+      </c>
+      <c r="H2">
+        <v>160494</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="B10" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>